<commit_message>
NOT READY TO PULL All college data (except cutoff) done Cutoff done till KKWIER for CAP 2025 Schema changes in document not fully modified models.py not modified yet
</commit_message>
<xml_diff>
--- a/data/cleaned_data/nashik_cleaned_data.xlsx
+++ b/data/cleaned_data/nashik_cleaned_data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="placement_stats" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="college_details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="branches" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +449,11 @@
           <t>avg_package</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -464,8 +470,6 @@
       <c r="D2" t="n">
         <v>2025</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -482,8 +486,6 @@
       <c r="D3" t="n">
         <v>2024</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -500,8 +502,6 @@
       <c r="D4" t="n">
         <v>2023</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -518,7 +518,6 @@
       <c r="D5" t="n">
         <v>2025</v>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>2</v>
       </c>
@@ -538,7 +537,6 @@
       <c r="D6" t="n">
         <v>2024</v>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
         <v>2</v>
       </c>
@@ -558,7 +556,6 @@
       <c r="D7" t="n">
         <v>2023</v>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>2</v>
       </c>
@@ -600,7 +597,6 @@
       <c r="D9" t="n">
         <v>2024</v>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>5.5</v>
       </c>
@@ -620,7 +616,6 @@
       <c r="D10" t="n">
         <v>2023</v>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
         <v>5.97</v>
       </c>
@@ -640,7 +635,6 @@
       <c r="D11" t="n">
         <v>2025</v>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
         <v>3</v>
       </c>
@@ -660,8 +654,6 @@
       <c r="D12" t="n">
         <v>2024</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -678,8 +670,6 @@
       <c r="D13" t="n">
         <v>2023</v>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -696,9 +686,13 @@
       <c r="D14" t="n">
         <v>2025</v>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
         <v>4.2</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -716,8 +710,6 @@
       <c r="D15" t="n">
         <v>2024</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -734,7 +726,6 @@
       <c r="D16" t="n">
         <v>2023</v>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
         <v>2.93</v>
       </c>
@@ -754,8 +745,6 @@
       <c r="D17" t="n">
         <v>2025</v>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -816,8 +805,6 @@
       <c r="D20" t="n">
         <v>2025</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -878,8 +865,6 @@
       <c r="D23" t="n">
         <v>2025</v>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -940,8 +925,6 @@
       <c r="D26" t="n">
         <v>2025</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1068,8 +1051,6 @@
       <c r="D32" t="n">
         <v>2025</v>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1130,8 +1111,6 @@
       <c r="D35" t="n">
         <v>2025</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1192,8 +1171,6 @@
       <c r="D38" t="n">
         <v>2025</v>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1248,7 +1225,6 @@
           <t>SUN</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
         <v>2025</v>
       </c>
@@ -1268,7 +1244,6 @@
           <t>SUN</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
         <v>2024</v>
       </c>
@@ -1288,7 +1263,6 @@
           <t>SUN</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="n">
         <v>2023</v>
       </c>
@@ -1380,8 +1354,6 @@
       <c r="D47" t="n">
         <v>2025</v>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1508,8 +1480,6 @@
       <c r="D53" t="n">
         <v>2025</v>
       </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1526,8 +1496,6 @@
       <c r="D54" t="n">
         <v>2024</v>
       </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1544,8 +1512,6 @@
       <c r="D55" t="n">
         <v>2023</v>
       </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1562,8 +1528,6 @@
       <c r="D56" t="n">
         <v>2025</v>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3027,7 +2991,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Varvandi / Dindori</t>
+          <t>Varvandi</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -3200,7 +3164,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Sinnar</t>
+          <t>Chincholi</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3447,6 +3411,4544 @@
       <c r="T20" t="n">
         <v>2013</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H151"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>branch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>college_abbrv</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>dte_code</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>branch_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>branch_abbrv</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>regular_intake</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>estimated_dse_intake</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>dse_intake_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>INTEGER
+(nn)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>VARCHAR
+(NN)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>VARCHAR
+(nn)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>VARCHAR
+(N)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BVCERI</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5130</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BVCERI</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5130</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BVCERI</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5130</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>60</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BVCERI</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5130</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>120</v>
+      </c>
+      <c r="G6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H6" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>120</v>
+      </c>
+      <c r="G7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>120</v>
+      </c>
+      <c r="G8" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H9" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>60</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>23</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>46</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>E&amp;C</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>60</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>JIT</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5401</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>60</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>120</v>
+      </c>
+      <c r="G15" t="n">
+        <v>12</v>
+      </c>
+      <c r="H15" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>120</v>
+      </c>
+      <c r="G16" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>120</v>
+      </c>
+      <c r="G17" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>120</v>
+      </c>
+      <c r="G18" t="n">
+        <v>12</v>
+      </c>
+      <c r="H18" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>120</v>
+      </c>
+      <c r="G19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H19" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CHEM</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>60</v>
+      </c>
+      <c r="G20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>120</v>
+      </c>
+      <c r="G21" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Robotics &amp; Automation Engineering</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>R&amp;A</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>120</v>
+      </c>
+      <c r="G22" t="n">
+        <v>12</v>
+      </c>
+      <c r="H22" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>120</v>
+      </c>
+      <c r="G23" t="n">
+        <v>12</v>
+      </c>
+      <c r="H23" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Computer Science and Design</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CSD</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>120</v>
+      </c>
+      <c r="G24" t="n">
+        <v>12</v>
+      </c>
+      <c r="H24" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LOGMIEER</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5390</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>60</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LOGMIEER</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5390</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>60</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>LOGMIEER</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>5390</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>30</v>
+      </c>
+      <c r="G27" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LOGMIEER</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>5390</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>60</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LOGMIEER</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>5390</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>60</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LOGMIEER</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>5390</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>AIML</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>60</v>
+      </c>
+      <c r="G30" t="n">
+        <v>6</v>
+      </c>
+      <c r="H30" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>LGNSCCOE</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>5182</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>120</v>
+      </c>
+      <c r="G31" t="n">
+        <v>12</v>
+      </c>
+      <c r="H31" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LGNSCCOE</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>5182</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>120</v>
+      </c>
+      <c r="G32" t="n">
+        <v>12</v>
+      </c>
+      <c r="H32" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>LGNSCCOE</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>5182</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>60</v>
+      </c>
+      <c r="G33" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>LGNSCCOE</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>5182</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>60</v>
+      </c>
+      <c r="G34" t="n">
+        <v>6</v>
+      </c>
+      <c r="H34" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LGNSCCOE</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>5182</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>120</v>
+      </c>
+      <c r="G35" t="n">
+        <v>12</v>
+      </c>
+      <c r="H35" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LGNSCCOE</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>5182</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>60</v>
+      </c>
+      <c r="G36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H36" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SNJB</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>5173</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>126</v>
+      </c>
+      <c r="G37" t="n">
+        <v>12</v>
+      </c>
+      <c r="H37" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SNJB</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>5173</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>63</v>
+      </c>
+      <c r="G38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SNJB</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5173</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>180</v>
+      </c>
+      <c r="G39" t="n">
+        <v>18</v>
+      </c>
+      <c r="H39" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SNJB</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>5173</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>63</v>
+      </c>
+      <c r="G40" t="n">
+        <v>6</v>
+      </c>
+      <c r="H40" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SNJB</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>5173</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>63</v>
+      </c>
+      <c r="G41" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>120</v>
+      </c>
+      <c r="G42" t="n">
+        <v>12</v>
+      </c>
+      <c r="H42" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>60</v>
+      </c>
+      <c r="G43" t="n">
+        <v>6</v>
+      </c>
+      <c r="H43" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>180</v>
+      </c>
+      <c r="G44" t="n">
+        <v>18</v>
+      </c>
+      <c r="H44" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>60</v>
+      </c>
+      <c r="G45" t="n">
+        <v>6</v>
+      </c>
+      <c r="H45" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>120</v>
+      </c>
+      <c r="G46" t="n">
+        <v>12</v>
+      </c>
+      <c r="H46" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>E&amp;C</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>120</v>
+      </c>
+      <c r="G47" t="n">
+        <v>12</v>
+      </c>
+      <c r="H47" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>120</v>
+      </c>
+      <c r="G48" t="n">
+        <v>12</v>
+      </c>
+      <c r="H48" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MCOERC</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>5177</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>60</v>
+      </c>
+      <c r="G49" t="n">
+        <v>6</v>
+      </c>
+      <c r="H49" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>120</v>
+      </c>
+      <c r="G50" t="n">
+        <v>12</v>
+      </c>
+      <c r="H50" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>120</v>
+      </c>
+      <c r="G51" t="n">
+        <v>12</v>
+      </c>
+      <c r="H51" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>120</v>
+      </c>
+      <c r="G52" t="n">
+        <v>12</v>
+      </c>
+      <c r="H52" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>60</v>
+      </c>
+      <c r="G53" t="n">
+        <v>6</v>
+      </c>
+      <c r="H53" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>120</v>
+      </c>
+      <c r="G54" t="n">
+        <v>12</v>
+      </c>
+      <c r="H54" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>60</v>
+      </c>
+      <c r="G55" t="n">
+        <v>6</v>
+      </c>
+      <c r="H55" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>60</v>
+      </c>
+      <c r="G56" t="n">
+        <v>6</v>
+      </c>
+      <c r="H56" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>METIOE</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>5151</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>E&amp;C</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>60</v>
+      </c>
+      <c r="G57" t="n">
+        <v>6</v>
+      </c>
+      <c r="H57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>120</v>
+      </c>
+      <c r="G58" t="n">
+        <v>12</v>
+      </c>
+      <c r="H58" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>180</v>
+      </c>
+      <c r="G59" t="n">
+        <v>18</v>
+      </c>
+      <c r="H59" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Instrumentation &amp; Control Engineering</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>60</v>
+      </c>
+      <c r="G60" t="n">
+        <v>6</v>
+      </c>
+      <c r="H60" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>120</v>
+      </c>
+      <c r="G61" t="n">
+        <v>12</v>
+      </c>
+      <c r="H61" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>120</v>
+      </c>
+      <c r="G62" t="n">
+        <v>12</v>
+      </c>
+      <c r="H62" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>180</v>
+      </c>
+      <c r="G63" t="n">
+        <v>18</v>
+      </c>
+      <c r="H63" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>180</v>
+      </c>
+      <c r="G64" t="n">
+        <v>18</v>
+      </c>
+      <c r="H64" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>60</v>
+      </c>
+      <c r="G65" t="n">
+        <v>6</v>
+      </c>
+      <c r="H65" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>KBTCOE</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5108</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>120</v>
+      </c>
+      <c r="G66" t="n">
+        <v>12</v>
+      </c>
+      <c r="H66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>PVGCOE</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5330</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>60</v>
+      </c>
+      <c r="G67" t="n">
+        <v>6</v>
+      </c>
+      <c r="H67" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>PVGCOE</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>5330</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>60</v>
+      </c>
+      <c r="G68" t="n">
+        <v>6</v>
+      </c>
+      <c r="H68" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>PVGCOE</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5330</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>60</v>
+      </c>
+      <c r="G69" t="n">
+        <v>6</v>
+      </c>
+      <c r="H69" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>PVGCOE</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>5330</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>60</v>
+      </c>
+      <c r="G70" t="n">
+        <v>6</v>
+      </c>
+      <c r="H70" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>PVGCOE</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>5330</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>60</v>
+      </c>
+      <c r="G71" t="n">
+        <v>6</v>
+      </c>
+      <c r="H71" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>RHSCOEMSR</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>5181</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>60</v>
+      </c>
+      <c r="G72" t="n">
+        <v>6</v>
+      </c>
+      <c r="H72" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>RHSCOEMSR</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>5181</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>60</v>
+      </c>
+      <c r="G73" t="n">
+        <v>6</v>
+      </c>
+      <c r="H73" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>RHSCOEMSR</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>5181</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>120</v>
+      </c>
+      <c r="G74" t="n">
+        <v>12</v>
+      </c>
+      <c r="H74" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>RHSCOEMSR</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>5181</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>120</v>
+      </c>
+      <c r="G75" t="n">
+        <v>12</v>
+      </c>
+      <c r="H75" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>RHSCOEMSR</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>5181</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>120</v>
+      </c>
+      <c r="G76" t="n">
+        <v>12</v>
+      </c>
+      <c r="H76" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>RHSCOEMSR</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>5181</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>120</v>
+      </c>
+      <c r="G77" t="n">
+        <v>12</v>
+      </c>
+      <c r="H77" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>60</v>
+      </c>
+      <c r="G78" t="n">
+        <v>6</v>
+      </c>
+      <c r="H78" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>180</v>
+      </c>
+      <c r="G79" t="n">
+        <v>18</v>
+      </c>
+      <c r="H79" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>60</v>
+      </c>
+      <c r="G80" t="n">
+        <v>6</v>
+      </c>
+      <c r="H80" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>120</v>
+      </c>
+      <c r="G81" t="n">
+        <v>12</v>
+      </c>
+      <c r="H81" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>120</v>
+      </c>
+      <c r="G82" t="n">
+        <v>12</v>
+      </c>
+      <c r="H82" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>60</v>
+      </c>
+      <c r="G83" t="n">
+        <v>6</v>
+      </c>
+      <c r="H83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>60</v>
+      </c>
+      <c r="G84" t="n">
+        <v>6</v>
+      </c>
+      <c r="H84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SIEM</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>5331</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>60</v>
+      </c>
+      <c r="G85" t="n">
+        <v>6</v>
+      </c>
+      <c r="H85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>60</v>
+      </c>
+      <c r="G86" t="n">
+        <v>6</v>
+      </c>
+      <c r="H86" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>120</v>
+      </c>
+      <c r="G87" t="n">
+        <v>12</v>
+      </c>
+      <c r="H87" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>60</v>
+      </c>
+      <c r="G88" t="n">
+        <v>6</v>
+      </c>
+      <c r="H88" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>60</v>
+      </c>
+      <c r="G89" t="n">
+        <v>6</v>
+      </c>
+      <c r="H89" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>60</v>
+      </c>
+      <c r="G90" t="n">
+        <v>6</v>
+      </c>
+      <c r="H90" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>60</v>
+      </c>
+      <c r="G91" t="n">
+        <v>6</v>
+      </c>
+      <c r="H91" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>60</v>
+      </c>
+      <c r="G92" t="n">
+        <v>6</v>
+      </c>
+      <c r="H92" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>60</v>
+      </c>
+      <c r="G93" t="n">
+        <v>6</v>
+      </c>
+      <c r="H93" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>AIML</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>60</v>
+      </c>
+      <c r="G94" t="n">
+        <v>6</v>
+      </c>
+      <c r="H94" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SITRC</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>5109</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>60</v>
+      </c>
+      <c r="G95" t="n">
+        <v>6</v>
+      </c>
+      <c r="H95" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Computer Science &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>120</v>
+      </c>
+      <c r="G96" t="n">
+        <v>12</v>
+      </c>
+      <c r="H96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>AIML</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>60</v>
+      </c>
+      <c r="G97" t="n">
+        <v>6</v>
+      </c>
+      <c r="H97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>60</v>
+      </c>
+      <c r="G98" t="n">
+        <v>6</v>
+      </c>
+      <c r="H98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Cloud Technology &amp; Information Security</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>CTIS</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>30</v>
+      </c>
+      <c r="G99" t="n">
+        <v>3</v>
+      </c>
+      <c r="H99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>98</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Cyber Security &amp; Forensics</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>CSF</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>30</v>
+      </c>
+      <c r="G100" t="n">
+        <v>3</v>
+      </c>
+      <c r="H100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>99</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Full Stack Development &amp; Testing (with AI &amp; ML)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>FSDT</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>30</v>
+      </c>
+      <c r="G101" t="n">
+        <v>3</v>
+      </c>
+      <c r="H101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>100</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Robotics Process Automation</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>30</v>
+      </c>
+      <c r="G102" t="n">
+        <v>3</v>
+      </c>
+      <c r="H102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Virtual &amp; Augmented Reality</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>VRAR</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>30</v>
+      </c>
+      <c r="G103" t="n">
+        <v>3</v>
+      </c>
+      <c r="H103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>102</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Aerospace Engineering</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>AES</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>30</v>
+      </c>
+      <c r="G104" t="n">
+        <v>3</v>
+      </c>
+      <c r="H104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>103</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Aeronautical Engineering</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>AEN</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>30</v>
+      </c>
+      <c r="G105" t="n">
+        <v>3</v>
+      </c>
+      <c r="H105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>104</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>60</v>
+      </c>
+      <c r="G106" t="n">
+        <v>6</v>
+      </c>
+      <c r="H106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>105</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>60</v>
+      </c>
+      <c r="G107" t="n">
+        <v>6</v>
+      </c>
+      <c r="H107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>106</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>30</v>
+      </c>
+      <c r="G108" t="n">
+        <v>3</v>
+      </c>
+      <c r="H108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>107</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>30</v>
+      </c>
+      <c r="G109" t="n">
+        <v>3</v>
+      </c>
+      <c r="H109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>108</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Biomedical Engineering</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>30</v>
+      </c>
+      <c r="G110" t="n">
+        <v>3</v>
+      </c>
+      <c r="H110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>109</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>BT</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>30</v>
+      </c>
+      <c r="G111" t="n">
+        <v>3</v>
+      </c>
+      <c r="H111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>110</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>5399</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>60</v>
+      </c>
+      <c r="G112" t="n">
+        <v>6</v>
+      </c>
+      <c r="H112" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>111</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>5399</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>60</v>
+      </c>
+      <c r="G113" t="n">
+        <v>6</v>
+      </c>
+      <c r="H113" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>112</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>5399</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>AIML</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>60</v>
+      </c>
+      <c r="G114" t="n">
+        <v>6</v>
+      </c>
+      <c r="H114" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>113</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>5399</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>60</v>
+      </c>
+      <c r="G115" t="n">
+        <v>6</v>
+      </c>
+      <c r="H115" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>114</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>5399</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>60</v>
+      </c>
+      <c r="G116" t="n">
+        <v>6</v>
+      </c>
+      <c r="H116" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>115</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>5399</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>60</v>
+      </c>
+      <c r="G117" t="n">
+        <v>6</v>
+      </c>
+      <c r="H117" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>116</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SIER</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>60</v>
+      </c>
+      <c r="G118" t="n">
+        <v>6</v>
+      </c>
+      <c r="H118" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>117</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SIER</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>60</v>
+      </c>
+      <c r="G119" t="n">
+        <v>6</v>
+      </c>
+      <c r="H119" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>118</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>SIER</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>60</v>
+      </c>
+      <c r="G120" t="n">
+        <v>6</v>
+      </c>
+      <c r="H120" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>119</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>SIER</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Electrionics &amp; Telecommunication Engineering</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>E&amp;TC</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>60</v>
+      </c>
+      <c r="G121" t="n">
+        <v>6</v>
+      </c>
+      <c r="H121" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>120</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SIER</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>60</v>
+      </c>
+      <c r="G122" t="n">
+        <v>6</v>
+      </c>
+      <c r="H122" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>121</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SVIT</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>5125</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>60</v>
+      </c>
+      <c r="G123" t="n">
+        <v>6</v>
+      </c>
+      <c r="H123" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>122</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>SVIT</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>5125</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>CHEM</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>60</v>
+      </c>
+      <c r="G124" t="n">
+        <v>6</v>
+      </c>
+      <c r="H124" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>123</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>SVIT</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>5125</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>E&amp;C</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>60</v>
+      </c>
+      <c r="G125" t="n">
+        <v>6</v>
+      </c>
+      <c r="H125" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>124</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>SVIT</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>5125</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>60</v>
+      </c>
+      <c r="G126" t="n">
+        <v>6</v>
+      </c>
+      <c r="H126" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>125</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>120</v>
+      </c>
+      <c r="G127" t="n">
+        <v>12</v>
+      </c>
+      <c r="H127" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>126</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>60</v>
+      </c>
+      <c r="G128" t="n">
+        <v>6</v>
+      </c>
+      <c r="H128" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>127</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>60</v>
+      </c>
+      <c r="G129" t="n">
+        <v>6</v>
+      </c>
+      <c r="H129" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>128</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>60</v>
+      </c>
+      <c r="G130" t="n">
+        <v>6</v>
+      </c>
+      <c r="H130" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>129</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Electronics &amp; Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>E&amp;C</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>60</v>
+      </c>
+      <c r="G131" t="n">
+        <v>6</v>
+      </c>
+      <c r="H131" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>130</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Mechatronics Engineering</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>60</v>
+      </c>
+      <c r="G132" t="n">
+        <v>6</v>
+      </c>
+      <c r="H132" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>131</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>SNDCOERC</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>5124</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>60</v>
+      </c>
+      <c r="G133" t="n">
+        <v>6</v>
+      </c>
+      <c r="H133" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>132</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>GCOERC</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>5418</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>120</v>
+      </c>
+      <c r="G134" t="n">
+        <v>12</v>
+      </c>
+      <c r="H134" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>133</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>GCOERC</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>5418</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>60</v>
+      </c>
+      <c r="G135" t="n">
+        <v>6</v>
+      </c>
+      <c r="H135" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>134</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>GCOERC</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>5418</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>60</v>
+      </c>
+      <c r="G136" t="n">
+        <v>6</v>
+      </c>
+      <c r="H136" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>135</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>GCOERC</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>5418</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>120</v>
+      </c>
+      <c r="G137" t="n">
+        <v>12</v>
+      </c>
+      <c r="H137" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>136</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>GCOERC</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>5418</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>60</v>
+      </c>
+      <c r="G138" t="n">
+        <v>6</v>
+      </c>
+      <c r="H138" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>137</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>GCOERC</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>5418</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>60</v>
+      </c>
+      <c r="G139" t="n">
+        <v>6</v>
+      </c>
+      <c r="H139" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>138</v>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>139</v>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>140</v>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>141</v>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>143</v>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" t="inlineStr"/>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" t="inlineStr"/>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Modified cleaning scripts, created a common file to execute all scripts
</commit_message>
<xml_diff>
--- a/data/cleaned_data/nashik_cleaned_data.xlsx
+++ b/data/cleaned_data/nashik_cleaned_data.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,11 +449,6 @@
           <t>avg_package</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Unnamed: 6</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -470,6 +465,8 @@
       <c r="D2" t="n">
         <v>2025</v>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -486,6 +483,8 @@
       <c r="D3" t="n">
         <v>2024</v>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -502,6 +501,8 @@
       <c r="D4" t="n">
         <v>2023</v>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -518,6 +519,7 @@
       <c r="D5" t="n">
         <v>2025</v>
       </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>2</v>
       </c>
@@ -537,6 +539,7 @@
       <c r="D6" t="n">
         <v>2024</v>
       </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
         <v>2</v>
       </c>
@@ -556,6 +559,7 @@
       <c r="D7" t="n">
         <v>2023</v>
       </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>2</v>
       </c>
@@ -597,6 +601,7 @@
       <c r="D9" t="n">
         <v>2024</v>
       </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>5.5</v>
       </c>
@@ -616,6 +621,7 @@
       <c r="D10" t="n">
         <v>2023</v>
       </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
         <v>5.97</v>
       </c>
@@ -635,6 +641,7 @@
       <c r="D11" t="n">
         <v>2025</v>
       </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
         <v>3</v>
       </c>
@@ -654,6 +661,8 @@
       <c r="D12" t="n">
         <v>2024</v>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -670,6 +679,8 @@
       <c r="D13" t="n">
         <v>2023</v>
       </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -686,13 +697,9 @@
       <c r="D14" t="n">
         <v>2025</v>
       </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
         <v>4.2</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
       </c>
     </row>
     <row r="15">
@@ -710,6 +717,8 @@
       <c r="D15" t="n">
         <v>2024</v>
       </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -726,6 +735,7 @@
       <c r="D16" t="n">
         <v>2023</v>
       </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
         <v>2.93</v>
       </c>
@@ -745,6 +755,8 @@
       <c r="D17" t="n">
         <v>2025</v>
       </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -805,6 +817,8 @@
       <c r="D20" t="n">
         <v>2025</v>
       </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -865,6 +879,8 @@
       <c r="D23" t="n">
         <v>2025</v>
       </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -925,6 +941,8 @@
       <c r="D26" t="n">
         <v>2025</v>
       </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1051,6 +1069,8 @@
       <c r="D32" t="n">
         <v>2025</v>
       </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1111,6 +1131,8 @@
       <c r="D35" t="n">
         <v>2025</v>
       </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1171,6 +1193,8 @@
       <c r="D38" t="n">
         <v>2025</v>
       </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1225,6 +1249,7 @@
           <t>SUN</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
         <v>2025</v>
       </c>
@@ -1244,6 +1269,7 @@
           <t>SUN</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
         <v>2024</v>
       </c>
@@ -1263,6 +1289,7 @@
           <t>SUN</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="n">
         <v>2023</v>
       </c>
@@ -1354,6 +1381,8 @@
       <c r="D47" t="n">
         <v>2025</v>
       </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1480,6 +1509,8 @@
       <c r="D53" t="n">
         <v>2025</v>
       </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1496,6 +1527,8 @@
       <c r="D54" t="n">
         <v>2024</v>
       </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1512,6 +1545,8 @@
       <c r="D55" t="n">
         <v>2023</v>
       </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1528,6 +1563,8 @@
       <c r="D56" t="n">
         <v>2025</v>
       </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3423,7 +3460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3469,38 +3506,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>INTEGER
-(nn)</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VARCHAR
-(NN)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>BVCERI</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5130</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>VARCHAR
-(nn)</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>VARCHAR
-(N)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>CIVIL</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>60</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -3512,12 +3551,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -3527,12 +3566,12 @@
         <v>6</v>
       </c>
       <c r="H3" t="n">
-        <v>39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -3544,12 +3583,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -3559,12 +3598,12 @@
         <v>6</v>
       </c>
       <c r="H4" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -3576,44 +3615,44 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H5" t="n">
-        <v>24</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BVCERI</t>
+          <t>JIT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5130</v>
+        <v>5401</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -3623,12 +3662,12 @@
         <v>12</v>
       </c>
       <c r="H6" t="n">
-        <v>114</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -3640,12 +3679,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -3655,12 +3694,12 @@
         <v>12</v>
       </c>
       <c r="H7" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -3672,12 +3711,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -3687,12 +3726,12 @@
         <v>12</v>
       </c>
       <c r="H8" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -3704,27 +3743,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G9" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H9" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -3736,27 +3775,27 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H10" t="n">
-        <v>47</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -3768,27 +3807,27 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H11" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -3800,27 +3839,27 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electronic &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>E&amp;C</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="G12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H12" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -3832,12 +3871,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Electronic &amp; Computer Engineering</t>
+          <t>Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>E&amp;C</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -3846,43 +3885,42 @@
       <c r="G13" t="n">
         <v>6</v>
       </c>
-      <c r="H13" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>KKWIER</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5121</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>COMP</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>120</v>
+      </c>
+      <c r="G14" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>JIT</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>5401</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Automation &amp; Robotics</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>60</v>
-      </c>
-      <c r="G14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -3894,12 +3932,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electronic &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -3909,12 +3947,12 @@
         <v>12</v>
       </c>
       <c r="H15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -3926,12 +3964,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Electronic &amp; Telecommunication Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -3941,12 +3979,12 @@
         <v>12</v>
       </c>
       <c r="H16" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -3958,12 +3996,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -3973,12 +4011,12 @@
         <v>12</v>
       </c>
       <c r="H17" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -3990,12 +4028,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -4005,12 +4043,12 @@
         <v>12</v>
       </c>
       <c r="H18" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -4022,27 +4060,27 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G19" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" t="n">
         <v>12</v>
-      </c>
-      <c r="H19" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -4054,27 +4092,27 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G20" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H20" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -4086,12 +4124,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Robotics &amp; Automation Engineering</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>R&amp;A</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -4101,12 +4139,12 @@
         <v>12</v>
       </c>
       <c r="H21" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -4118,12 +4156,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Robotics &amp; Automation Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>R&amp;A</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -4133,12 +4171,12 @@
         <v>12</v>
       </c>
       <c r="H22" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -4150,12 +4188,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Computer Science and Design</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -4165,44 +4203,44 @@
         <v>12</v>
       </c>
       <c r="H23" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KKWIER</t>
+          <t>LOGMIEER</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5121</v>
+        <v>5390</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Computer Science and Design</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H24" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -4214,12 +4252,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -4229,12 +4267,12 @@
         <v>6</v>
       </c>
       <c r="H25" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -4246,27 +4284,27 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H26" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -4278,27 +4316,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H27" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -4310,12 +4348,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -4325,12 +4363,12 @@
         <v>6</v>
       </c>
       <c r="H28" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -4342,12 +4380,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>AIML</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -4357,44 +4395,44 @@
         <v>6</v>
       </c>
       <c r="H29" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LOGMIEER</t>
+          <t>LGNSCCOE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>5390</v>
+        <v>5182</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Machine Learning</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AIML</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G30" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H30" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -4406,12 +4444,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -4421,12 +4459,12 @@
         <v>12</v>
       </c>
       <c r="H31" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -4438,27 +4476,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G32" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H32" t="n">
-        <v>16</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -4470,12 +4508,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -4485,12 +4523,12 @@
         <v>6</v>
       </c>
       <c r="H33" t="n">
-        <v>45</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -4502,27 +4540,27 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G34" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H34" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -4534,59 +4572,59 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G35" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H35" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>LGNSCCOE</t>
+          <t>SNJB</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>5182</v>
+        <v>5173</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="G36" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H36" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -4598,27 +4636,27 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="G37" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H37" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -4630,27 +4668,27 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>63</v>
+        <v>180</v>
       </c>
       <c r="G38" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H38" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -4662,27 +4700,27 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electronics &amp; Telecommunication</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>180</v>
+        <v>63</v>
       </c>
       <c r="G39" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H39" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -4694,12 +4732,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -4709,44 +4747,44 @@
         <v>6</v>
       </c>
       <c r="H40" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SNJB</t>
+          <t>MCOERC</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>5173</v>
+        <v>5177</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="G41" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H41" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -4758,27 +4796,27 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G42" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H42" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -4790,27 +4828,27 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="G43" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H43" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -4822,27 +4860,27 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="G44" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H44" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -4854,27 +4892,27 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G45" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H45" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -4886,12 +4924,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Electronics &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>E&amp;C</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -4901,12 +4939,12 @@
         <v>12</v>
       </c>
       <c r="H46" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -4918,12 +4956,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Electronics &amp; Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>E&amp;C</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -4933,12 +4971,12 @@
         <v>12</v>
       </c>
       <c r="H47" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -4950,59 +4988,59 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G48" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H48" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MCOERC</t>
+          <t>METIOE</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>5177</v>
+        <v>5151</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G49" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H49" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -5014,12 +5052,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -5029,12 +5067,12 @@
         <v>12</v>
       </c>
       <c r="H50" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -5046,12 +5084,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -5061,12 +5099,12 @@
         <v>12</v>
       </c>
       <c r="H51" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -5078,27 +5116,27 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G52" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H52" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -5110,27 +5148,27 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G53" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H53" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -5142,27 +5180,27 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G54" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H54" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -5174,12 +5212,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -5194,7 +5232,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -5206,12 +5244,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electronics &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>E&amp;C</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -5220,43 +5258,42 @@
       <c r="G56" t="n">
         <v>6</v>
       </c>
-      <c r="H56" t="n">
-        <v>16</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>METIOE</t>
+          <t>KBTCOE</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>5151</v>
+        <v>5108</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Electronics &amp; Computer Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>E&amp;C</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G57" t="n">
-        <v>6</v>
-      </c>
-      <c r="H57" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="H57" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -5268,27 +5305,27 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="G58" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H58" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -5300,27 +5337,27 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Instrumentation &amp; Control Engineering</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="G59" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H59" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -5332,19 +5369,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; Control Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G60" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H60" t="n">
         <v>13</v>
@@ -5352,7 +5389,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -5364,12 +5401,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -5379,12 +5416,12 @@
         <v>12</v>
       </c>
       <c r="H61" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -5396,19 +5433,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="G62" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H62" t="n">
         <v>15</v>
@@ -5416,7 +5453,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -5428,12 +5465,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -5443,12 +5480,12 @@
         <v>18</v>
       </c>
       <c r="H63" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -5460,19 +5497,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="G64" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H64" t="n">
         <v>17</v>
@@ -5480,7 +5517,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -5492,57 +5529,56 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G65" t="n">
-        <v>6</v>
-      </c>
-      <c r="H65" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>KBTCOE</t>
+          <t>PVGCOE</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>5108</v>
+        <v>5330</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Automation &amp; Robotics</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G66" t="n">
-        <v>12</v>
-      </c>
-      <c r="H66" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="H66" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -5554,12 +5590,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -5569,12 +5605,12 @@
         <v>6</v>
       </c>
       <c r="H67" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -5586,12 +5622,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -5606,7 +5642,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -5618,12 +5654,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -5633,12 +5669,12 @@
         <v>6</v>
       </c>
       <c r="H69" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -5650,12 +5686,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -5665,29 +5701,29 @@
         <v>6</v>
       </c>
       <c r="H70" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PVGCOE</t>
+          <t>RHSCOEMSR</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5330</v>
+        <v>5181</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -5697,12 +5733,12 @@
         <v>6</v>
       </c>
       <c r="H71" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -5714,12 +5750,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -5729,12 +5765,12 @@
         <v>6</v>
       </c>
       <c r="H72" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -5746,27 +5782,27 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G73" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H73" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -5778,12 +5814,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -5793,12 +5829,12 @@
         <v>12</v>
       </c>
       <c r="H74" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -5810,12 +5846,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -5825,12 +5861,12 @@
         <v>12</v>
       </c>
       <c r="H75" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -5842,12 +5878,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -5857,44 +5893,44 @@
         <v>12</v>
       </c>
       <c r="H76" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RHSCOEMSR</t>
+          <t>SIEM</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>5181</v>
+        <v>5331</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G77" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H77" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -5906,27 +5942,27 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="G78" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H78" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -5938,27 +5974,27 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="G79" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H79" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -5970,27 +6006,27 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G80" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H80" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -6002,12 +6038,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -6017,12 +6053,12 @@
         <v>12</v>
       </c>
       <c r="H81" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -6034,27 +6070,24 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G82" t="n">
-        <v>12</v>
-      </c>
-      <c r="H82" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -6066,12 +6099,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -6080,11 +6113,10 @@
       <c r="G83" t="n">
         <v>6</v>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6096,12 +6128,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -6110,28 +6142,27 @@
       <c r="G84" t="n">
         <v>6</v>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SIEM</t>
+          <t>SITRC</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>5331</v>
+        <v>5109</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Automation &amp; Robotics</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -6140,11 +6171,13 @@
       <c r="G85" t="n">
         <v>6</v>
       </c>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -6156,27 +6189,27 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G86" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H86" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -6188,27 +6221,27 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G87" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H87" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -6220,12 +6253,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -6235,12 +6268,12 @@
         <v>6</v>
       </c>
       <c r="H88" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -6252,12 +6285,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -6267,12 +6300,12 @@
         <v>6</v>
       </c>
       <c r="H89" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -6284,12 +6317,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -6304,7 +6337,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -6316,12 +6349,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -6331,12 +6364,12 @@
         <v>6</v>
       </c>
       <c r="H91" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -6348,12 +6381,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -6363,12 +6396,12 @@
         <v>6</v>
       </c>
       <c r="H92" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -6380,12 +6413,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Automation &amp; Robotics</t>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AIML</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -6395,12 +6428,12 @@
         <v>6</v>
       </c>
       <c r="H93" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -6412,12 +6445,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Machine Learning</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>AIML</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -6427,87 +6460,78 @@
         <v>6</v>
       </c>
       <c r="H94" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SITRC</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>5109</v>
+          <t>SUN</t>
+        </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Computer Science &amp; Engineering</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>CSE</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G95" t="n">
-        <v>6</v>
-      </c>
-      <c r="H95" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Computer Science &amp; Engineering</t>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>CSE</t>
+          <t>AIML</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G96" t="n">
-        <v>12</v>
-      </c>
-      <c r="H96" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Machine Learning</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>AIML</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -6516,54 +6540,50 @@
       <c r="G97" t="n">
         <v>6</v>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Cloud Technology &amp; Information Security</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>CTIS</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G98" t="n">
-        <v>6</v>
-      </c>
-      <c r="H98" t="inlineStr"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Cloud Technology &amp; Information Security</t>
+          <t>Cyber Security &amp; Forensics</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>CTIS</t>
+          <t>CSF</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -6572,26 +6592,24 @@
       <c r="G99" t="n">
         <v>3</v>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Cyber Security &amp; Forensics</t>
+          <t>Full Stack Development &amp; Testing (with AI &amp; ML)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>CSF</t>
+          <t>FSDT</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -6600,26 +6618,24 @@
       <c r="G100" t="n">
         <v>3</v>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Full Stack Development &amp; Testing (with AI &amp; ML)</t>
+          <t>Robotics Process Automation</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>FSDT</t>
+          <t>RPA</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -6628,26 +6644,24 @@
       <c r="G101" t="n">
         <v>3</v>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Robotics Process Automation</t>
+          <t>Virtual &amp; Augmented Reality</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>RPA</t>
+          <t>VRAR</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -6656,26 +6670,24 @@
       <c r="G102" t="n">
         <v>3</v>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Virtual &amp; Augmented Reality</t>
+          <t>Aerospace Engineering</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>VRAR</t>
+          <t>AES</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -6684,26 +6696,24 @@
       <c r="G103" t="n">
         <v>3</v>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Aerospace Engineering</t>
+          <t>Aeronautical Engineering</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>AES</t>
+          <t>AEN</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -6712,54 +6722,50 @@
       <c r="G104" t="n">
         <v>3</v>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Aeronautical Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>AEN</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="G105" t="n">
-        <v>3</v>
-      </c>
-      <c r="H105" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -6768,54 +6774,50 @@
       <c r="G106" t="n">
         <v>6</v>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G107" t="n">
-        <v>6</v>
-      </c>
-      <c r="H107" t="inlineStr"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Electronics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -6824,26 +6826,24 @@
       <c r="G108" t="n">
         <v>3</v>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Electronics &amp; Telecommunication Engineering</t>
+          <t>Biomedical Engineering</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>BME</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -6852,26 +6852,24 @@
       <c r="G109" t="n">
         <v>3</v>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
           <t>SUN</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Biomedical Engineering</t>
+          <t>Biotechnology</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>BME</t>
+          <t>BT</t>
         </is>
       </c>
       <c r="F110" t="n">
@@ -6880,39 +6878,42 @@
       <c r="G110" t="n">
         <v>3</v>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SUN</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr"/>
+          <t>SCOE</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>5399</v>
+      </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Biotechnology</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F111" t="n">
+        <v>60</v>
+      </c>
+      <c r="G111" t="n">
+        <v>6</v>
+      </c>
+      <c r="H111" t="n">
         <v>30</v>
       </c>
-      <c r="G111" t="n">
-        <v>3</v>
-      </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -6924,12 +6925,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F112" t="n">
@@ -6939,12 +6940,12 @@
         <v>6</v>
       </c>
       <c r="H112" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -6956,12 +6957,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>AIML</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -6971,12 +6972,12 @@
         <v>6</v>
       </c>
       <c r="H113" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -6988,12 +6989,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Machine Learning</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>AIML</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -7003,12 +7004,12 @@
         <v>6</v>
       </c>
       <c r="H114" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -7020,12 +7021,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F115" t="n">
@@ -7035,12 +7036,12 @@
         <v>6</v>
       </c>
       <c r="H115" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -7052,12 +7053,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F116" t="n">
@@ -7067,29 +7068,29 @@
         <v>6</v>
       </c>
       <c r="H116" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SCOE</t>
+          <t>SIER</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>5399</v>
+        <v>5184</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -7099,12 +7100,12 @@
         <v>6</v>
       </c>
       <c r="H117" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -7116,12 +7117,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -7131,12 +7132,12 @@
         <v>6</v>
       </c>
       <c r="H118" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -7148,12 +7149,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -7163,12 +7164,12 @@
         <v>6</v>
       </c>
       <c r="H119" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -7180,12 +7181,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Electrionics &amp; Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>E&amp;TC</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -7195,12 +7196,12 @@
         <v>6</v>
       </c>
       <c r="H120" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -7212,12 +7213,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Electrionics &amp; Telecommunication Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>E&amp;TC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -7227,29 +7228,29 @@
         <v>6</v>
       </c>
       <c r="H121" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SIER</t>
+          <t>SVIT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>5184</v>
+        <v>5125</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -7259,12 +7260,12 @@
         <v>6</v>
       </c>
       <c r="H122" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -7276,12 +7277,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>CHEM</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -7291,12 +7292,12 @@
         <v>6</v>
       </c>
       <c r="H123" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -7308,12 +7309,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Electronics &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>CHEM</t>
+          <t>E&amp;C</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -7323,12 +7324,12 @@
         <v>6</v>
       </c>
       <c r="H124" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -7340,12 +7341,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Electronics &amp; Computer Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>E&amp;C</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -7355,44 +7356,44 @@
         <v>6</v>
       </c>
       <c r="H125" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SVIT</t>
+          <t>SNDCOERC</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>5125</v>
+        <v>5124</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G126" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H126" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -7404,27 +7405,27 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G127" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H127" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -7436,12 +7437,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -7451,12 +7452,12 @@
         <v>6</v>
       </c>
       <c r="H128" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -7468,12 +7469,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -7483,12 +7484,12 @@
         <v>6</v>
       </c>
       <c r="H129" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -7500,12 +7501,12 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Electronics &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>E&amp;C</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -7515,12 +7516,12 @@
         <v>6</v>
       </c>
       <c r="H130" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -7532,12 +7533,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Electronics &amp; Computer Engineering</t>
+          <t>Mechatronics Engineering</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>E&amp;C</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -7547,12 +7548,12 @@
         <v>6</v>
       </c>
       <c r="H131" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -7564,12 +7565,12 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Mechatronics Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -7579,44 +7580,44 @@
         <v>6</v>
       </c>
       <c r="H132" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SNDCOERC</t>
+          <t>GCOERC</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>5124</v>
+        <v>5418</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Artificial Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G133" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H133" t="n">
-        <v>58</v>
+        <v>8</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -7628,27 +7629,27 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Artificial Intelligence &amp; Data Science</t>
+          <t>Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G134" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H134" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -7660,12 +7661,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Automation &amp; Robotics</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CIVIL</t>
         </is>
       </c>
       <c r="F135" t="n">
@@ -7675,12 +7676,12 @@
         <v>6</v>
       </c>
       <c r="H135" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -7692,27 +7693,27 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Computer Engineering</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>CIVIL</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G136" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H136" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -7724,27 +7725,27 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G137" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H137" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -7756,12 +7757,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>MECH</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -7771,184 +7772,8 @@
         <v>6</v>
       </c>
       <c r="H138" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="n">
-        <v>137</v>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>GCOERC</t>
-        </is>
-      </c>
-      <c r="C139" t="n">
-        <v>5418</v>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>Mechanical Engineering</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>MECH</t>
-        </is>
-      </c>
-      <c r="F139" t="n">
-        <v>60</v>
-      </c>
-      <c r="G139" t="n">
-        <v>6</v>
-      </c>
-      <c r="H139" t="n">
         <v>23</v>
       </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="n">
-        <v>138</v>
-      </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
-      <c r="D140" t="inlineStr"/>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
-      <c r="H140" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" t="n">
-        <v>139</v>
-      </c>
-      <c r="B141" t="inlineStr"/>
-      <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr"/>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
-      <c r="H141" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" t="n">
-        <v>140</v>
-      </c>
-      <c r="B142" t="inlineStr"/>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr"/>
-      <c r="H142" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" t="n">
-        <v>141</v>
-      </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
-      <c r="H143" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" t="n">
-        <v>142</v>
-      </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
-      <c r="H144" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" t="n">
-        <v>143</v>
-      </c>
-      <c r="B145" t="inlineStr"/>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr"/>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
-      <c r="H145" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" t="n">
-        <v>144</v>
-      </c>
-      <c r="B146" t="inlineStr"/>
-      <c r="C146" t="inlineStr"/>
-      <c r="D146" t="inlineStr"/>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr"/>
-      <c r="H146" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" t="n">
-        <v>145</v>
-      </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" t="n">
-        <v>146</v>
-      </c>
-      <c r="B148" t="inlineStr"/>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" t="n">
-        <v>147</v>
-      </c>
-      <c r="B149" t="inlineStr"/>
-      <c r="C149" t="inlineStr"/>
-      <c r="D149" t="inlineStr"/>
-      <c r="E149" t="inlineStr"/>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>148</v>
-      </c>
-      <c r="B150" t="inlineStr"/>
-      <c r="C150" t="inlineStr"/>
-      <c r="D150" t="inlineStr"/>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
-      <c r="H150" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="n">
-        <v>149</v>
-      </c>
-      <c r="B151" t="inlineStr"/>
-      <c r="C151" t="inlineStr"/>
-      <c r="D151" t="inlineStr"/>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
-      <c r="H151" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Wrote data loading scripts, and successfully loaded data into LOCAL DB
</commit_message>
<xml_diff>
--- a/data/cleaned_data/nashik_cleaned_data.xlsx
+++ b/data/cleaned_data/nashik_cleaned_data.xlsx
@@ -2910,71 +2910,69 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B15" t="n">
+        <v>5399</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sandip University</t>
+          <t>S.M.E.S. Sanghavi College of Engineering</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SUN</t>
+          <t>SCOE</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Gut No. 166, Mhasrul-Varvandi Road, Varvandi, Taluka Dindori - 422202</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Varvandi</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Nashik</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Sandip University, Mahiravani, Tal &amp; Dist: Nashik - 422213, Trambakeshwar Rd, Nashik, Maharashtra 422213</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Mahiravani</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Nashik</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2(f)</t>
-        </is>
-      </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>18002122714</t>
+          <t>02532307630</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2988,32 +2986,32 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>9.130000000000001</v>
+        <v>2.9</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://www.sandipuniversity.edu.in/</t>
+          <t>https://engineering.shreemahavir.org/</t>
         </is>
       </c>
       <c r="T15" t="n">
-        <v>2017</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" t="n">
-        <v>5399</v>
+        <v>5184</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>S.M.E.S. Sanghavi College of Engineering</t>
+          <t>Shatabdi Institute of Engineering and Research</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SCOE</t>
+          <t>SIER</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3023,12 +3021,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Gut No. 166, Mhasrul-Varvandi Road, Varvandi, Taluka Dindori - 422202</t>
+          <t>RR8J+68C, Agaskhind, (Via Deolali Camp - Bhagur), Post-Shenit, Tal, Dist, Sinnar, Maharashtra 422502</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Varvandi</t>
+          <t>Sinnar</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -3046,11 +3044,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3063,12 +3056,12 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>02532307630</t>
+          <t>02551304203</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -3077,32 +3070,32 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>https://engineering.shreemahavir.org/</t>
+          <t>https://siernashik.org.in/</t>
         </is>
       </c>
       <c r="T16" t="n">
-        <v>2012</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" t="n">
-        <v>5184</v>
+        <v>5125</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shatabdi Institute of Engineering and Research</t>
+          <t>Sir Visvesvaraya Institute of Technology</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SIER</t>
+          <t>SVIT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3112,12 +3105,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RR8J+68C, Agaskhind, (Via Deolali Camp - Bhagur), Post-Shenit, Tal, Dist, Sinnar, Maharashtra 422502</t>
+          <t>A/P Chincholi, Taluka Sinnar, Nashik - 422102</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Sinnar</t>
+          <t>Chincholi</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -3135,6 +3128,11 @@
           <t>no</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3142,17 +3140,22 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2(f)</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>02551304203</t>
+          <t>9423787347</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -3161,32 +3164,32 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>2.6</v>
+        <v>2.97</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>https://siernashik.org.in/</t>
+          <t>https://svitnashik.in/</t>
         </is>
       </c>
       <c r="T17" t="n">
-        <v>2009</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18" t="n">
-        <v>5125</v>
+        <v>5124</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sir Visvesvaraya Institute of Technology</t>
+          <t>SND College of Engineering and Research Center</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SVIT</t>
+          <t>SNDCOERC</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3196,12 +3199,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>A/P Chincholi, Taluka Sinnar, Nashik - 422102</t>
+          <t>Lasalgaon Patoda Yeola Rd, Yeola, Babhulgaon Bk., Maharashtra 423401, India</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Chincholi</t>
+          <t>Yeola</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3216,12 +3219,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>B++</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -3241,7 +3244,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>9423787347</t>
+          <t>2559225011</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -3255,32 +3258,32 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>2.97</v>
+        <v>2.56</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>https://svitnashik.in/</t>
+          <t>https://sndcoe.ac.in/</t>
         </is>
       </c>
       <c r="T18" t="n">
-        <v>1998</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" t="n">
-        <v>5124</v>
+        <v>5418</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SND College of Engineering and Research Center</t>
+          <t>Guru Gobind Singh College Of Engineering And Research Centre, Nashik</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SNDCOERC</t>
+          <t>GCOERC</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3290,12 +3293,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Lasalgaon Patoda Yeola Rd, Yeola, Babhulgaon Bk., Maharashtra 423401, India</t>
+          <t>Khalsa Educational Complex Guru Gobind Singh Marg, Wadala-Parhardi Road,, Annexe Nashik,, Indira Nagar, Nashik, Maharashtra 422102</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yeola</t>
+          <t>Nashik</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -3310,12 +3313,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>B++</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -3325,17 +3328,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>2(f)</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2559225011</t>
+          <t>7768004583</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -3349,54 +3347,51 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>2.56</v>
+        <v>3.16</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>https://sndcoe.ac.in/</t>
+          <t>https://engg.ggsf.edu.in/</t>
         </is>
       </c>
       <c r="T19" t="n">
-        <v>2006</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="n">
-        <v>5418</v>
+        <v>14</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Guru Gobind Singh College Of Engineering And Research Centre, Nashik</t>
+          <t>Sandip University</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GCOERC</t>
+          <t>SUN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Khalsa Educational Complex Guru Gobind Singh Marg, Wadala-Parhardi Road,, Annexe Nashik,, Indira Nagar, Nashik, Maharashtra 422102</t>
+          <t>Sandip University, Mahiravani, Tal &amp; Dist: Nashik - 422213, Trambakeshwar Rd, Nashik, Maharashtra 422213</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>Mahiravani</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>Nashik</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Nashik</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>Private</t>
@@ -3404,27 +3399,32 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2(f)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>7768004583</t>
+          <t>18002122714</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -3438,15 +3438,15 @@
         </is>
       </c>
       <c r="R20" t="n">
-        <v>3.16</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>https://engg.ggsf.edu.in/</t>
+          <t>https://www.sandipuniversity.edu.in/</t>
         </is>
       </c>
       <c r="T20" t="n">
-        <v>2013</v>
+        <v>2017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>